<commit_message>
v0.13: fix request formatting in Excel
Remove frozen panes (clipped the title and section names in column B), stop
merging the SR25 header across hidden columns I-K, widen column H.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
@@ -627,7 +627,7 @@
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
     <col hidden="1" width="16" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="50" customWidth="1" min="10" max="10"/>
     <col hidden="1" width="24" customWidth="1" min="11" max="11"/>
@@ -648,7 +648,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>End-2026 target status assessment and reporting (v0.12)</t>
+          <t>End-2026 target status assessment and reporting (v0.13)</t>
         </is>
       </c>
     </row>
@@ -756,7 +756,7 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>End-2025 reporting (click the ref to see your full SR25 response)</t>
+          <t>SR25 response</t>
         </is>
       </c>
       <c r="L13" s="13" t="inlineStr">
@@ -1154,9 +1154,8 @@
     <row r="20"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <mergeCells count="10">
+  <mergeCells count="9">
     <mergeCell ref="M7:N7"/>
-    <mergeCell ref="H13:K13"/>
     <mergeCell ref="B4:C8"/>
     <mergeCell ref="M6:N6"/>
     <mergeCell ref="L13:R13"/>

</xml_diff>

<commit_message>
v0.14: no target status rating in 2026
Remove the Met/Partially met/Not met column, its dropdown and definitions box
from every request (columns shift left by one), reword instructions and the
SR25 opening line. A1 becomes 'A1. Response summary' (units asked, responses
received, awaiting, owner confirmed); T1/T2, tracker counts, links, protection,
Read me, Issues log and project timeline updated. check.py guards against
rating text returning.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -78,18 +78,6 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Aptos"/>
-      <b val="1"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <i val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <name val="Aptos Narrow"/>
       <b val="1"/>
       <sz val="22"/>
@@ -125,8 +113,12 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <name val="Aptos"/>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -146,11 +138,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C1E4F5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -191,38 +178,31 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -234,13 +214,14 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -617,7 +598,7 @@
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R20"/>
+  <dimension ref="A1:Q20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -631,13 +612,12 @@
     <col hidden="1" width="16" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="50" customWidth="1" min="10" max="10"/>
     <col hidden="1" width="24" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="48" customWidth="1" min="12" max="12"/>
     <col width="48" customWidth="1" min="13" max="13"/>
-    <col width="48" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -648,303 +628,231 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>End-2026 target status assessment and reporting (v0.13)</t>
+          <t>SR26 sustainability reporting (v0.14)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>End-2026 target status confirmation and reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>Target status assessment and definitions</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="B4" s="5" t="inlineStr">
+          <t>SR26 sustainability reporting request</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>How to use this spreadsheet:</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>• Confirm target status for each row below (Column L). Refer to target status definitions to the right for guidance.
-• Provide commentary on progress towards each target (Column M or N)
-• Provide supporting documentation if required (Column O), including links to images
-• Note the source of your information and any limitations (Column P), then confirm the information is accurate (Columns Q–R)
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>• For each row below, describe progress towards the target (Column L) and/or respond to the 2026 reporting request (Column M)
+• Provide supporting information if required (Column N), including links to documents or images
+• Note the source of your information and any limitations (Column O), then confirm the information is accurate (Columns P–Q)
 • Where a related end-2025 target existed, click the ref in Column H to see your full SR25 response (Tab 3)
 • Use Tab 2 of this spreadsheet to highlight key sustainability stories (optional)
-• 2026 is a transition year: Sustainability 2030 launched ~20 October 2026, so report on activity across all of 2026 and any early actions since launch.
+• 2026 is a transition year: Sustainability 2030 launched ~20 October 2026, so report on activity across all of 2026 and any early actions since launch. No target status rating is requested this year.
 • Due: Tuesday 15 December 2026. Questions: CDSS – questions and clarifications are recorded centrally (contact email TBC); optional 1:1 meetings available on request</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>Met or exceeded</t>
-        </is>
-      </c>
-      <c r="M4" s="8" t="inlineStr">
-        <is>
-          <t>The data and information provided demonstrates that the Faculty/Portfolio has met or exceeded the target</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="32" customHeight="1">
-      <c r="L5" s="7" t="inlineStr">
-        <is>
-          <t>Partially met</t>
-        </is>
-      </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>The data and information provided indicates that the target has not been met, but there has been a significant improvement and performance is trending towards the target</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="32" customHeight="1">
-      <c r="L6" s="7" t="inlineStr">
-        <is>
-          <t>Not met</t>
-        </is>
-      </c>
-      <c r="M6" s="8" t="inlineStr">
-        <is>
-          <t>Some action has been taken to address the target, but the data and information provided demonstrates that this has been insufficient to meet the target</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="32" customHeight="1">
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>Not yet started</t>
-        </is>
-      </c>
-      <c r="M7" s="8" t="inlineStr">
-        <is>
-          <t>No action has been taken.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="L8" s="9" t="n"/>
-    </row>
-    <row r="9">
-      <c r="L9" s="10" t="inlineStr">
-        <is>
-          <t>Note: target status definitions are under review for 2027 reporting. 2026 ratings are for internal management reporting only.</t>
-        </is>
-      </c>
-    </row>
+    </row>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8" ht="60" customHeight="1"/>
     <row r="11">
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>AC&amp;M – Advancement, Communication and Marketing</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Sustainability 2030 target and indicator</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>SR25 response</t>
         </is>
       </c>
-      <c r="L13" s="13" t="inlineStr">
+      <c r="L13" s="8" t="inlineStr">
         <is>
           <t>End-2026 reporting (PLEASE COMPLETE THIS SECTION)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Priority area</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Sustainability 2030 target</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>2026 Reporting request</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G14" s="9" t="inlineStr">
         <is>
           <t>How SST will use this data</t>
         </is>
       </c>
-      <c r="H14" s="14" t="inlineStr">
+      <c r="H14" s="9" t="inlineStr">
         <is>
           <t>Related SR25 ref</t>
         </is>
       </c>
-      <c r="I14" s="14" t="inlineStr">
+      <c r="I14" s="9" t="inlineStr">
         <is>
           <t>End-2025 confirmed status</t>
         </is>
       </c>
-      <c r="J14" s="14" t="inlineStr">
+      <c r="J14" s="9" t="inlineStr">
         <is>
           <t>End-2025 reporting response</t>
         </is>
       </c>
-      <c r="K14" s="14" t="inlineStr">
+      <c r="K14" s="9" t="inlineStr">
         <is>
           <t>Links and supporting information</t>
         </is>
       </c>
-      <c r="L14" s="15" t="inlineStr">
-        <is>
-          <t>Confirm end-2026 target status</t>
-        </is>
-      </c>
-      <c r="M14" s="15" t="inlineStr">
+      <c r="L14" s="10" t="inlineStr">
         <is>
           <t>OPTION 1:  Target-level reporting (Column D)</t>
         </is>
       </c>
-      <c r="N14" s="15" t="inlineStr">
+      <c r="M14" s="10" t="inlineStr">
         <is>
           <t>OPTION 2:  Indicator level reporting (Column E/F)</t>
         </is>
       </c>
-      <c r="O14" s="15" t="inlineStr">
+      <c r="N14" s="10" t="inlineStr">
         <is>
           <t>Supporting information/comments</t>
         </is>
       </c>
-      <c r="P14" s="15" t="inlineStr">
+      <c r="O14" s="10" t="inlineStr">
         <is>
           <t>Data source and limitations</t>
         </is>
       </c>
-      <c r="Q14" s="15" t="inlineStr">
+      <c r="P14" s="10" t="inlineStr">
         <is>
           <t>Data owner confirms information is accurate</t>
         </is>
       </c>
-      <c r="R14" s="15" t="inlineStr">
+      <c r="Q14" s="10" t="inlineStr">
         <is>
           <t>Confirmed by (name, role, date)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="16" t="inlineStr"/>
-      <c r="C15" s="16" t="inlineStr"/>
-      <c r="D15" s="16" t="inlineStr"/>
-      <c r="E15" s="16" t="inlineStr"/>
-      <c r="F15" s="16" t="inlineStr"/>
-      <c r="G15" s="16" t="inlineStr"/>
-      <c r="H15" s="16" t="inlineStr"/>
-      <c r="I15" s="16" t="inlineStr"/>
-      <c r="J15" s="16" t="inlineStr"/>
-      <c r="K15" s="16" t="inlineStr"/>
-      <c r="L15" s="16" t="inlineStr">
-        <is>
-          <t>(Met or exceeded; partially met; not met; not yet started)</t>
-        </is>
-      </c>
-      <c r="M15" s="16" t="inlineStr">
-        <is>
-          <t>Provide further evidence of target status assessment in the form of:
-A general update on activities in relation to the overarching target (Column D)</t>
-        </is>
-      </c>
-      <c r="N15" s="16" t="inlineStr">
-        <is>
-          <t>Provide further evidence of target status assessment in the form of:
-Data and commentary in direct response to the reporting request (Column F)</t>
-        </is>
-      </c>
-      <c r="O15" s="16" t="inlineStr">
-        <is>
-          <t>Provide any additional information to support the target status assessment (e.g. links, images, rationale for selection of target status)</t>
-        </is>
-      </c>
-      <c r="P15" s="16" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr"/>
+      <c r="C15" s="11" t="inlineStr"/>
+      <c r="D15" s="11" t="inlineStr"/>
+      <c r="E15" s="11" t="inlineStr"/>
+      <c r="F15" s="11" t="inlineStr"/>
+      <c r="G15" s="11" t="inlineStr"/>
+      <c r="H15" s="11" t="inlineStr"/>
+      <c r="I15" s="11" t="inlineStr"/>
+      <c r="J15" s="11" t="inlineStr"/>
+      <c r="K15" s="11" t="inlineStr"/>
+      <c r="L15" s="11" t="inlineStr">
+        <is>
+          <t>A general update on activities in relation to the overarching target (Column D)</t>
+        </is>
+      </c>
+      <c r="M15" s="11" t="inlineStr">
+        <is>
+          <t>Data and commentary in direct response to the reporting request (Column F)</t>
+        </is>
+      </c>
+      <c r="N15" s="11" t="inlineStr">
+        <is>
+          <t>Any additional information (e.g. links, images, documents)</t>
+        </is>
+      </c>
+      <c r="O15" s="11" t="inlineStr">
         <is>
           <t>Where did this information come from (system, report, survey, person)? Note any gaps or limitations.</t>
         </is>
       </c>
-      <c r="Q15" s="16" t="inlineStr">
+      <c r="P15" s="11" t="inlineStr">
         <is>
           <t>Select 'Yes' to confirm the information provided is accurate and can be used for reporting</t>
         </is>
       </c>
-      <c r="R15" s="16" t="inlineStr">
+      <c r="Q15" s="11" t="inlineStr">
         <is>
           <t>Name, role and date of the person confirming</t>
         </is>
       </c>
     </row>
     <row r="16" ht="150" customHeight="1">
-      <c r="B16" s="17" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>TR2(a)</t>
         </is>
       </c>
-      <c r="C16" s="18" t="inlineStr">
+      <c r="C16" s="13" t="inlineStr">
         <is>
           <t>Transformational research</t>
         </is>
       </c>
-      <c r="D16" s="18" t="inlineStr">
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
         </is>
       </c>
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes</t>
         </is>
       </c>
-      <c r="F16" s="19" t="inlineStr">
-        <is>
-          <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) and rated it 'Met or exceeded' (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
+      <c r="F16" s="14" t="inlineStr">
+        <is>
+          <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
 Please provide examples of sustainability-related research impact from your Faculty/Portfolio across policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.</t>
         </is>
       </c>
-      <c r="G16" s="19" t="inlineStr">
+      <c r="G16" s="14" t="inlineStr">
         <is>
           <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from MRE.</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
+      <c r="H16" s="15" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I16" s="19" t="inlineStr">
+      <c r="I16" s="14" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J16" s="19" t="inlineStr">
+      <c r="J16" s="14" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -953,7 +861,7 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="K16" s="19" t="inlineStr">
+      <c r="K16" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -966,105 +874,103 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L16" s="21" t="n"/>
-      <c r="M16" s="21" t="n"/>
-      <c r="N16" s="21" t="n"/>
-      <c r="O16" s="21" t="n"/>
-      <c r="P16" s="21" t="n"/>
-      <c r="Q16" s="21" t="n"/>
-      <c r="R16" s="21" t="n"/>
+      <c r="L16" s="16" t="n"/>
+      <c r="M16" s="16" t="n"/>
+      <c r="N16" s="16" t="n"/>
+      <c r="O16" s="16" t="n"/>
+      <c r="P16" s="16" t="n"/>
+      <c r="Q16" s="16" t="n"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="B17" s="17" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>CL2(a)</t>
         </is>
       </c>
-      <c r="C17" s="18" t="inlineStr">
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>Climate leadership</t>
         </is>
       </c>
-      <c r="D17" s="18" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Develop understanding of our research and education programs that contribute to accelerating global decarbonisation and our own climate transition.</t>
         </is>
       </c>
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>By 2028, develop and document institutional mapping of research and education activities that are designed to contribute to global decarbonisation</t>
         </is>
       </c>
-      <c r="F17" s="19" t="inlineStr">
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>Please list and describe examples of communications from your Faculty/Portfolio that demonstrate climate action, research and learning and aim to inform policy, sector or community decarbonisation efforts. Could include links, intended audiences and any available evidence of reach or influence.</t>
         </is>
       </c>
-      <c r="G17" s="19" t="inlineStr">
+      <c r="G17" s="14" t="inlineStr">
         <is>
           <t>We will use these examples to show how the University communicates climate research and learning to external audiences, and as an input to the institutional decarbonisation research and education mapping due by 2028.</t>
         </is>
       </c>
-      <c r="H17" s="19" t="inlineStr">
+      <c r="H17" s="14" t="inlineStr">
         <is>
           <t>N/A – new indicator</t>
         </is>
       </c>
-      <c r="I17" s="19" t="inlineStr"/>
-      <c r="J17" s="19" t="inlineStr"/>
-      <c r="K17" s="19" t="inlineStr"/>
-      <c r="L17" s="21" t="n"/>
-      <c r="M17" s="21" t="n"/>
-      <c r="N17" s="21" t="n"/>
-      <c r="O17" s="21" t="n"/>
-      <c r="P17" s="21" t="n"/>
-      <c r="Q17" s="21" t="n"/>
-      <c r="R17" s="21" t="n"/>
+      <c r="I17" s="14" t="inlineStr"/>
+      <c r="J17" s="14" t="inlineStr"/>
+      <c r="K17" s="14" t="inlineStr"/>
+      <c r="L17" s="16" t="n"/>
+      <c r="M17" s="16" t="n"/>
+      <c r="N17" s="16" t="n"/>
+      <c r="O17" s="16" t="n"/>
+      <c r="P17" s="16" t="n"/>
+      <c r="Q17" s="16" t="n"/>
     </row>
     <row r="18" ht="150" customHeight="1">
-      <c r="B18" s="17" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>CL2(c)</t>
         </is>
       </c>
-      <c r="C18" s="18" t="inlineStr">
+      <c r="C18" s="13" t="inlineStr">
         <is>
           <t>Climate leadership</t>
         </is>
       </c>
-      <c r="D18" s="18" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Develop understanding of our research and education programs that contribute to accelerating global decarbonisation and our own climate transition.</t>
         </is>
       </c>
-      <c r="E18" s="18" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>Ongoing communications that evidence the University’s climate action, research and learning to inform policy, sector and community decarbonisation efforts.</t>
         </is>
       </c>
-      <c r="F18" s="19" t="inlineStr">
-        <is>
-          <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) and rated it 'Met or exceeded' (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
 List and describe communications from the faculty in terms of climate action, research and learning to inform policy, sector and community decarbonisation efforts</t>
         </is>
       </c>
-      <c r="G18" s="19" t="inlineStr">
+      <c r="G18" s="14" t="inlineStr">
         <is>
           <t>We will report on the University's ongoing climate communications in the Climate leadership section of the 2026 Sustainability Report, alongside contributions from Melbourne Climate Futures and the Melbourne Energy Institute.</t>
         </is>
       </c>
-      <c r="H18" s="20" t="inlineStr">
+      <c r="H18" s="15" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I18" s="19" t="inlineStr">
+      <c r="I18" s="14" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J18" s="19" t="inlineStr">
+      <c r="J18" s="14" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -1073,7 +979,7 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="K18" s="19" t="inlineStr">
+      <c r="K18" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -1086,90 +992,80 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L18" s="21" t="n"/>
-      <c r="M18" s="21" t="n"/>
-      <c r="N18" s="21" t="n"/>
-      <c r="O18" s="21" t="n"/>
-      <c r="P18" s="21" t="n"/>
-      <c r="Q18" s="21" t="n"/>
-      <c r="R18" s="21" t="n"/>
+      <c r="L18" s="16" t="n"/>
+      <c r="M18" s="16" t="n"/>
+      <c r="N18" s="16" t="n"/>
+      <c r="O18" s="16" t="n"/>
+      <c r="P18" s="16" t="n"/>
+      <c r="Q18" s="16" t="n"/>
     </row>
     <row r="19" ht="150" customHeight="1">
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>EN1(c)</t>
         </is>
       </c>
-      <c r="C19" s="18" t="inlineStr">
+      <c r="C19" s="13" t="inlineStr">
         <is>
           <t>Enablers</t>
         </is>
       </c>
-      <c r="D19" s="18" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>Enablers</t>
         </is>
       </c>
-      <c r="E19" s="18" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>Coordinated internal engagement and external partnerships contributing to delivery of sustainability outcomes across priority areas.</t>
         </is>
       </c>
-      <c r="F19" s="19" t="inlineStr">
-        <is>
-          <t>In end-2025 reporting your area reported on the related SP2030 target 3e and rated it 'Met or exceeded' (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>In end-2025 reporting your area reported on the related SP2030 target 3e (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
 Please provide examples of internal engagement or external partnerships involving your Faculty/Portfolio that contributed to Sustainability 2030 outcomes, could include the priority area addressed, participating groups/partners, nature of the collaboration and key outcomes.</t>
         </is>
       </c>
-      <c r="G19" s="19" t="inlineStr">
+      <c r="G19" s="14" t="inlineStr">
         <is>
           <t>We will report on internal engagement and partnerships contributing to Sustainability 2030 outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
         </is>
       </c>
-      <c r="H19" s="20" t="inlineStr">
+      <c r="H19" s="15" t="inlineStr">
         <is>
           <t>3e
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I19" s="19" t="inlineStr">
+      <c r="I19" s="14" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J19" s="19" t="inlineStr">
+      <c r="J19" s="14" t="inlineStr">
         <is>
           <t>A total of 1,947 alumni have attended one or more of the 70 climate or sustainability-related events so far this year, a small increase over the 2024 total.  Overall alumni engagement has declined slightly from last year, and so this result is encouraging.  Additional focus on impact in this space has been incorporated into the strategic planning activities for 2026 with the hopes of further widening and deepening engagement.</t>
         </is>
       </c>
-      <c r="K19" s="19" t="inlineStr"/>
-      <c r="L19" s="21" t="n"/>
-      <c r="M19" s="21" t="n"/>
-      <c r="N19" s="21" t="n"/>
-      <c r="O19" s="21" t="n"/>
-      <c r="P19" s="21" t="n"/>
-      <c r="Q19" s="21" t="n"/>
-      <c r="R19" s="21" t="n"/>
+      <c r="K19" s="14" t="inlineStr"/>
+      <c r="L19" s="16" t="n"/>
+      <c r="M19" s="16" t="n"/>
+      <c r="N19" s="16" t="n"/>
+      <c r="O19" s="16" t="n"/>
+      <c r="P19" s="16" t="n"/>
+      <c r="Q19" s="16" t="n"/>
     </row>
     <row r="20"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
-  <mergeCells count="9">
-    <mergeCell ref="M7:N7"/>
+  <mergeCells count="4">
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="L13:Q13"/>
+    <mergeCell ref="D4:G8"/>
     <mergeCell ref="B4:C8"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="L13:R13"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="D4:G8"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="L3:N3"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation sqref="L16:L19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
-      <formula1>=Lists!$B$3:$B$7</formula1>
-    </dataValidation>
-    <dataValidation sqref="Q16:Q19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
+  <dataValidations count="1">
+    <dataValidation sqref="P16:P19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
       <formula1>=Lists!$C$2:$C$4</formula1>
     </dataValidation>
   </dataValidations>
@@ -1211,7 +1107,7 @@
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <t>End-2026 target status assessment and reporting</t>
+          <t>SR26 sustainability reporting</t>
         </is>
       </c>
     </row>
@@ -1223,12 +1119,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>How to use this spreadsheet</t>
         </is>
       </c>
-      <c r="C5" s="22" t="inlineStr">
+      <c r="C5" s="18" t="inlineStr">
         <is>
           <t>Please share up to 3 stories from 2026 which highlight your faculty's/portfolio's sustainability progress and/or impact. These stories can directly relate to Sustainability 2030 targets and indicators, or sustainability more generally. Due: Tuesday 15 December 2026 (early submission helps us develop case studies).</t>
         </is>
@@ -1236,77 +1132,77 @@
     </row>
     <row r="6"/>
     <row r="8">
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="19" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="19" t="inlineStr">
         <is>
           <t>Related Sustainability 2030 targets (optional)</t>
         </is>
       </c>
-      <c r="E8" s="23" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>Images and other media</t>
         </is>
       </c>
-      <c r="F8" s="23" t="inlineStr">
+      <c r="F8" s="19" t="inlineStr">
         <is>
           <t>Links and supporting documentation</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="B9" s="24" t="inlineStr"/>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr"/>
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>• Please include a brief description of a project or activity that has made a significant contribution to sustainability at the University (up to 250 words)
 • Summarise the benefits. Benefits may relate to operational outcomes, environmental/social outcomes, and sector benefits.</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr"/>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr"/>
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>(link to OneDrive/SharePoint files or published online content preferred)</t>
         </is>
       </c>
-      <c r="F9" s="24" t="inlineStr"/>
+      <c r="F9" s="20" t="inlineStr"/>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="21" t="n"/>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="21" t="n"/>
-      <c r="E10" s="21" t="n"/>
-      <c r="F10" s="21" t="n"/>
+      <c r="B10" s="16" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="16" t="n"/>
+      <c r="E10" s="16" t="n"/>
+      <c r="F10" s="16" t="n"/>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="21" t="n"/>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="21" t="n"/>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="21" t="n"/>
+      <c r="B11" s="16" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="16" t="n"/>
+      <c r="E11" s="16" t="n"/>
+      <c r="F11" s="16" t="n"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="21" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
+      <c r="B12" s="16" t="n"/>
+      <c r="C12" s="16" t="n"/>
+      <c r="D12" s="16" t="n"/>
+      <c r="E12" s="16" t="n"/>
+      <c r="F12" s="16" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -1357,158 +1253,158 @@
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="B3" s="22" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Your responses to the end-2025 reporting request, against the former Sustainability Plan 2030 (SP2030) targets. For reference only – please do not edit. Use the 'Back to request' links to return to the reporting template.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>← Back to request</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="26" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Advancement, Communications &amp; Marketing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>SR25 ref</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>SP2030 target</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>2025 reporting request</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Confirmed end-2025 status</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>OPTION 1: Target-level reporting</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>OPTION 2: Indicator-level reporting</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>Supporting information/comments</t>
         </is>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
         <is>
           <t>Related SR26 indicator(s)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="160" customHeight="1">
-      <c r="B7" s="17" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>3e</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>The University has increased its engagement with alumni regarding sustainability</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
         <is>
           <t>Annual climate and sustainability alumni community snapshot, including the number of related events and high-level audience demographics</t>
         </is>
       </c>
-      <c r="E7" s="19" t="inlineStr">
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F7" s="19" t="inlineStr">
+      <c r="F7" s="14" t="inlineStr">
         <is>
           <t>A total of 1,947 alumni have attended one or more of the 70 climate or sustainability-related events so far this year, a small increase over the 2024 total.  Overall alumni engagement has declined slightly from last year, and so this result is encouraging.  Additional focus on impact in this space has been incorporated into the strategic planning activities for 2026 with the hopes of further widening and deepening engagement.</t>
         </is>
       </c>
-      <c r="G7" s="19" t="inlineStr"/>
-      <c r="H7" s="19" t="inlineStr"/>
-      <c r="I7" s="19" t="inlineStr">
+      <c r="G7" s="14" t="inlineStr"/>
+      <c r="H7" s="14" t="inlineStr"/>
+      <c r="I7" s="14" t="inlineStr">
         <is>
           <t>EN1(c)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="160" customHeight="1">
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>4b(iii)</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Graduates have increased capabilities to shape, lead and succeed in the careers, communities and industries of sustainable societies (year on year).</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Alumni Profile or case study demonstrating the impact our alumni have in sustainability is produced.</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F8" s="19" t="inlineStr">
+      <c r="F8" s="14" t="inlineStr">
         <is>
           <t>In the second half of 2025, there was 1 new article published on the Alumni website featuring University alumni that are having an impact on sustainability. The focus of the article was on nature and people and how the alum is helping to change behaviours to improve conservation efforts. The article was featured in the Alumni Newsletter and promoted on alumni social media.</t>
         </is>
       </c>
-      <c r="G8" s="19" t="inlineStr"/>
-      <c r="H8" s="19" t="inlineStr">
+      <c r="G8" s="14" t="inlineStr"/>
+      <c r="H8" s="14" t="inlineStr">
         <is>
           <t>https://www.unimelb.edu.au/alumni/stay-connected/news-and-stories/fast-five-with-whos-who-at-the-zoo</t>
         </is>
       </c>
-      <c r="I8" s="19" t="inlineStr"/>
+      <c r="I8" s="14" t="inlineStr"/>
     </row>
     <row r="9" ht="160" customHeight="1">
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>5b(ii)</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>The highest quality research is conducted that contributes to knowledge, action, and impact across the disciplinary and interdisciplinary dimensions of sustainability.</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>Commentary on use of communication channels to disseminate sustainability-related research externally and the translation of sustainability-related research outcomes internally, drawing on Academic Division-level plans and varied cross-divisional activities and related outputs</t>
         </is>
       </c>
-      <c r="E9" s="19" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F9" s="19" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -1517,8 +1413,8 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="G9" s="19" t="inlineStr"/>
-      <c r="H9" s="19" t="inlineStr">
+      <c r="G9" s="14" t="inlineStr"/>
+      <c r="H9" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -1531,7 +1427,7 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="I9" s="19" t="inlineStr">
+      <c r="I9" s="14" t="inlineStr">
         <is>
           <t>TR2(a), CL2(c)</t>
         </is>
@@ -1554,13 +1450,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:I9"/>
+  <dimension ref="B1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" t="inlineStr">
         <is>
-          <t>End 2026 target status</t>
+          <t>(not used – no target status rating in 2026)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1576,21 +1472,6 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>Y/N</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Target status</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Score</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Response count</t>
         </is>
       </c>
     </row>
@@ -1615,24 +1496,8 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Met or exceeded</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="3">
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Met or exceeded</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1648,24 +1513,8 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Partially met</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="4">
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Partially met</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>Partially – see comments</t>
@@ -1681,47 +1530,15 @@
           <t>TBC</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Not met</t>
-        </is>
-      </c>
-      <c r="H4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Not met</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
           <t>Received</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Not yet started</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Not yet started</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>First review</t>
@@ -1729,11 +1546,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
         <is>
           <t>Follow-up</t>

</xml_diff>

<commit_message>
v0.17: Excel-online formatting pass on every workbook
Remove the row-1 running header and version (version kept in file properties),
freeze header rows only so titles are never clipped, size rows to wrapped text
(headers, explanation rows, request text), taller title row. check.py enforces
the layout rules on every visible request sheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
@@ -20,21 +20,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Aptos"/>
-      <color rgb="00002060"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Aptos"/>
@@ -178,61 +170,59 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -620,32 +610,22 @@
     <col width="24" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>↑</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>SR26 sustainability reporting (v0.16)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="3" t="inlineStr">
+    <row r="1"/>
+    <row r="2" ht="39" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>SR26 sustainability reporting request</t>
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>How to use this spreadsheet:</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>• For each row below, describe progress towards the target (Column L) and/or respond to the 2026 reporting request (Column M)
 • Provide supporting information if required (Column N), including links to documents or images
@@ -661,198 +641,201 @@
     <row r="6"/>
     <row r="7"/>
     <row r="8" ht="60" customHeight="1"/>
-    <row r="11">
-      <c r="B11" s="6" t="inlineStr">
+    <row r="9"/>
+    <row r="10"/>
+    <row r="11" ht="39" customHeight="1">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>AC&amp;M – Advancement, Communication and Marketing</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="C13" s="7" t="inlineStr">
+    <row r="12"/>
+    <row r="13" ht="27" customHeight="1">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Sustainability 2030 target and indicator</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
+      <c r="H13" s="5" t="inlineStr">
         <is>
           <t>SR25 response</t>
         </is>
       </c>
-      <c r="L13" s="8" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>End-2026 reporting (PLEASE COMPLETE THIS SECTION)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="9" t="inlineStr">
+    <row r="14" ht="60" customHeight="1">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Priority area</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Sustainability 2030 target</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>2026 Reporting request</t>
         </is>
       </c>
-      <c r="G14" s="9" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>How SST will use this data</t>
         </is>
       </c>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>Related SR25 ref</t>
         </is>
       </c>
-      <c r="I14" s="9" t="inlineStr">
+      <c r="I14" s="7" t="inlineStr">
         <is>
           <t>End-2025 confirmed status</t>
         </is>
       </c>
-      <c r="J14" s="9" t="inlineStr">
+      <c r="J14" s="7" t="inlineStr">
         <is>
           <t>End-2025 reporting response</t>
         </is>
       </c>
-      <c r="K14" s="9" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>Links and supporting information</t>
         </is>
       </c>
-      <c r="L14" s="10" t="inlineStr">
+      <c r="L14" s="8" t="inlineStr">
         <is>
           <t>OPTION 1:  Target-level reporting (Column D)</t>
         </is>
       </c>
-      <c r="M14" s="10" t="inlineStr">
+      <c r="M14" s="8" t="inlineStr">
         <is>
           <t>OPTION 2:  Indicator level reporting (Column E/F)</t>
         </is>
       </c>
-      <c r="N14" s="10" t="inlineStr">
+      <c r="N14" s="8" t="inlineStr">
         <is>
           <t>Supporting information/comments</t>
         </is>
       </c>
-      <c r="O14" s="10" t="inlineStr">
+      <c r="O14" s="8" t="inlineStr">
         <is>
           <t>Data source and limitations</t>
         </is>
       </c>
-      <c r="P14" s="10" t="inlineStr">
+      <c r="P14" s="8" t="inlineStr">
         <is>
           <t>Data owner confirms information is accurate</t>
         </is>
       </c>
-      <c r="Q14" s="10" t="inlineStr">
+      <c r="Q14" s="8" t="inlineStr">
         <is>
           <t>Confirmed by (name, role, date)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="11" t="inlineStr"/>
-      <c r="C15" s="11" t="inlineStr"/>
-      <c r="D15" s="11" t="inlineStr"/>
-      <c r="E15" s="11" t="inlineStr"/>
-      <c r="F15" s="11" t="inlineStr"/>
-      <c r="G15" s="11" t="inlineStr"/>
-      <c r="H15" s="11" t="inlineStr"/>
-      <c r="I15" s="11" t="inlineStr"/>
-      <c r="J15" s="11" t="inlineStr"/>
-      <c r="K15" s="11" t="inlineStr"/>
-      <c r="L15" s="11" t="inlineStr">
+    <row r="15" ht="81" customHeight="1">
+      <c r="B15" s="9" t="inlineStr"/>
+      <c r="C15" s="9" t="inlineStr"/>
+      <c r="D15" s="9" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr"/>
+      <c r="F15" s="9" t="inlineStr"/>
+      <c r="G15" s="9" t="inlineStr"/>
+      <c r="H15" s="9" t="inlineStr"/>
+      <c r="I15" s="9" t="inlineStr"/>
+      <c r="J15" s="9" t="inlineStr"/>
+      <c r="K15" s="9" t="inlineStr"/>
+      <c r="L15" s="9" t="inlineStr">
         <is>
           <t>A general update on activities in relation to the overarching target (Column D)</t>
         </is>
       </c>
-      <c r="M15" s="11" t="inlineStr">
+      <c r="M15" s="9" t="inlineStr">
         <is>
           <t>Data and commentary in direct response to the reporting request (Column F)</t>
         </is>
       </c>
-      <c r="N15" s="11" t="inlineStr">
+      <c r="N15" s="9" t="inlineStr">
         <is>
           <t>Any additional information (e.g. links, images, documents)</t>
         </is>
       </c>
-      <c r="O15" s="11" t="inlineStr">
+      <c r="O15" s="9" t="inlineStr">
         <is>
           <t>Where did this information come from (system, report, survey, person)? Note any gaps or limitations.</t>
         </is>
       </c>
-      <c r="P15" s="11" t="inlineStr">
+      <c r="P15" s="9" t="inlineStr">
         <is>
           <t>Select 'Yes' to confirm the information provided is accurate and can be used for reporting</t>
         </is>
       </c>
-      <c r="Q15" s="11" t="inlineStr">
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>Name, role and date of the person confirming</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="150" customHeight="1">
-      <c r="B16" s="12" t="inlineStr">
+    <row r="16" ht="204" customHeight="1">
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>TR2(a)</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>Transformational research</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
 Please provide examples of sustainability-related research impact from your Faculty/Portfolio across policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
+      <c r="G16" s="12" t="inlineStr">
         <is>
           <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from MRE.</t>
         </is>
       </c>
-      <c r="H16" s="15" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I16" s="14" t="inlineStr">
+      <c r="I16" s="12" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J16" s="14" t="inlineStr">
+      <c r="J16" s="12" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -861,7 +844,7 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="K16" s="14" t="inlineStr">
+      <c r="K16" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -874,103 +857,103 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L16" s="16" t="n"/>
-      <c r="M16" s="16" t="n"/>
-      <c r="N16" s="16" t="n"/>
-      <c r="O16" s="16" t="n"/>
-      <c r="P16" s="16" t="n"/>
-      <c r="Q16" s="16" t="n"/>
+      <c r="L16" s="14" t="n"/>
+      <c r="M16" s="14" t="n"/>
+      <c r="N16" s="14" t="n"/>
+      <c r="O16" s="14" t="n"/>
+      <c r="P16" s="14" t="n"/>
+      <c r="Q16" s="14" t="n"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="10" t="inlineStr">
         <is>
           <t>CL2(a)</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Climate leadership</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="11" t="inlineStr">
         <is>
           <t>Develop understanding of our research and education programs that contribute to accelerating global decarbonisation and our own climate transition.</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>By 2028, develop and document institutional mapping of research and education activities that are designed to contribute to global decarbonisation</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Please list and describe examples of communications from your Faculty/Portfolio that demonstrate climate action, research and learning and aim to inform policy, sector or community decarbonisation efforts. Could include links, intended audiences and any available evidence of reach or influence.</t>
         </is>
       </c>
-      <c r="G17" s="14" t="inlineStr">
+      <c r="G17" s="12" t="inlineStr">
         <is>
           <t>We will use these examples to show how the University communicates climate research and learning to external audiences, and as an input to the institutional decarbonisation research and education mapping due by 2028.</t>
         </is>
       </c>
-      <c r="H17" s="14" t="inlineStr">
+      <c r="H17" s="12" t="inlineStr">
         <is>
           <t>N/A – new indicator</t>
         </is>
       </c>
-      <c r="I17" s="14" t="inlineStr"/>
-      <c r="J17" s="14" t="inlineStr"/>
-      <c r="K17" s="14" t="inlineStr"/>
-      <c r="L17" s="16" t="n"/>
-      <c r="M17" s="16" t="n"/>
-      <c r="N17" s="16" t="n"/>
-      <c r="O17" s="16" t="n"/>
-      <c r="P17" s="16" t="n"/>
-      <c r="Q17" s="16" t="n"/>
-    </row>
-    <row r="18" ht="150" customHeight="1">
-      <c r="B18" s="12" t="inlineStr">
+      <c r="I17" s="12" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr"/>
+      <c r="K17" s="12" t="inlineStr"/>
+      <c r="L17" s="14" t="n"/>
+      <c r="M17" s="14" t="n"/>
+      <c r="N17" s="14" t="n"/>
+      <c r="O17" s="14" t="n"/>
+      <c r="P17" s="14" t="n"/>
+      <c r="Q17" s="14" t="n"/>
+    </row>
+    <row r="18" ht="171" customHeight="1">
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>CL2(c)</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>Climate leadership</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="11" t="inlineStr">
         <is>
           <t>Develop understanding of our research and education programs that contribute to accelerating global decarbonisation and our own climate transition.</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Ongoing communications that evidence the University’s climate action, research and learning to inform policy, sector and community decarbonisation efforts.</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
 List and describe communications from the faculty in terms of climate action, research and learning to inform policy, sector and community decarbonisation efforts</t>
         </is>
       </c>
-      <c r="G18" s="14" t="inlineStr">
+      <c r="G18" s="12" t="inlineStr">
         <is>
           <t>We will report on the University's ongoing climate communications in the Climate leadership section of the 2026 Sustainability Report, alongside contributions from Melbourne Climate Futures and the Melbourne Energy Institute.</t>
         </is>
       </c>
-      <c r="H18" s="15" t="inlineStr">
+      <c r="H18" s="13" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I18" s="14" t="inlineStr">
+      <c r="I18" s="12" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J18" s="14" t="inlineStr">
+      <c r="J18" s="12" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -979,7 +962,7 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="K18" s="14" t="inlineStr">
+      <c r="K18" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -992,68 +975,68 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L18" s="16" t="n"/>
-      <c r="M18" s="16" t="n"/>
-      <c r="N18" s="16" t="n"/>
-      <c r="O18" s="16" t="n"/>
-      <c r="P18" s="16" t="n"/>
-      <c r="Q18" s="16" t="n"/>
-    </row>
-    <row r="19" ht="150" customHeight="1">
-      <c r="B19" s="12" t="inlineStr">
+      <c r="L18" s="14" t="n"/>
+      <c r="M18" s="14" t="n"/>
+      <c r="N18" s="14" t="n"/>
+      <c r="O18" s="14" t="n"/>
+      <c r="P18" s="14" t="n"/>
+      <c r="Q18" s="14" t="n"/>
+    </row>
+    <row r="19" ht="188" customHeight="1">
+      <c r="B19" s="10" t="inlineStr">
         <is>
           <t>EN1(c)</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Enablers</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="D19" s="11" t="inlineStr">
         <is>
           <t>Enablers</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>Coordinated internal engagement and external partnerships contributing to delivery of sustainability outcomes across priority areas.</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="12" t="inlineStr">
         <is>
           <t>In end-2025 reporting your area reported on the related SP2030 target 3e (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
 Please provide examples of internal engagement or external partnerships involving your Faculty/Portfolio that contributed to Sustainability 2030 outcomes, could include the priority area addressed, participating groups/partners, nature of the collaboration and key outcomes.</t>
         </is>
       </c>
-      <c r="G19" s="14" t="inlineStr">
+      <c r="G19" s="12" t="inlineStr">
         <is>
           <t>We will report on internal engagement and partnerships contributing to Sustainability 2030 outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
         </is>
       </c>
-      <c r="H19" s="15" t="inlineStr">
+      <c r="H19" s="13" t="inlineStr">
         <is>
           <t>3e
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I19" s="14" t="inlineStr">
+      <c r="I19" s="12" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J19" s="14" t="inlineStr">
+      <c r="J19" s="12" t="inlineStr">
         <is>
           <t>A total of 1,947 alumni have attended one or more of the 70 climate or sustainability-related events so far this year, a small increase over the 2024 total.  Overall alumni engagement has declined slightly from last year, and so this result is encouraging.  Additional focus on impact in this space has been incorporated into the strategic planning activities for 2026 with the hopes of further widening and deepening engagement.</t>
         </is>
       </c>
-      <c r="K19" s="14" t="inlineStr"/>
-      <c r="L19" s="16" t="n"/>
-      <c r="M19" s="16" t="n"/>
-      <c r="N19" s="16" t="n"/>
-      <c r="O19" s="16" t="n"/>
-      <c r="P19" s="16" t="n"/>
-      <c r="Q19" s="16" t="n"/>
+      <c r="K19" s="12" t="inlineStr"/>
+      <c r="L19" s="14" t="n"/>
+      <c r="M19" s="14" t="n"/>
+      <c r="N19" s="14" t="n"/>
+      <c r="O19" s="14" t="n"/>
+      <c r="P19" s="14" t="n"/>
+      <c r="Q19" s="14" t="n"/>
     </row>
     <row r="20"/>
   </sheetData>
@@ -1099,110 +1082,102 @@
     <col width="30" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>↑</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>SR26 sustainability reporting</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="3" t="inlineStr">
+    <row r="1"/>
+    <row r="2" ht="39" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Highlighted stories (optional)</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="17" t="inlineStr">
+    <row r="3"/>
+    <row r="4"/>
+    <row r="5" ht="22" customHeight="1">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>How to use this spreadsheet</t>
         </is>
       </c>
-      <c r="C5" s="18" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Please share up to 3 stories from 2026 which highlight your faculty's/portfolio's sustainability progress and/or impact. These stories can directly relate to Sustainability 2030 targets and indicators, or sustainability more generally. Due: Tuesday 15 December 2026 (early submission helps us develop case studies).</t>
         </is>
       </c>
     </row>
     <row r="6"/>
-    <row r="8">
-      <c r="B8" s="19" t="inlineStr">
+    <row r="7"/>
+    <row r="8" ht="39" customHeight="1">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C8" s="19" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>Related Sustainability 2030 targets (optional)</t>
         </is>
       </c>
-      <c r="E8" s="19" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Images and other media</t>
         </is>
       </c>
-      <c r="F8" s="19" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>Links and supporting documentation</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="B9" s="20" t="inlineStr"/>
-      <c r="C9" s="20" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr"/>
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>• Please include a brief description of a project or activity that has made a significant contribution to sustainability at the University (up to 250 words)
 • Summarise the benefits. Benefits may relate to operational outcomes, environmental/social outcomes, and sector benefits.</t>
         </is>
       </c>
-      <c r="D9" s="20" t="inlineStr"/>
-      <c r="E9" s="20" t="inlineStr">
+      <c r="D9" s="18" t="inlineStr"/>
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>(link to OneDrive/SharePoint files or published online content preferred)</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr"/>
+      <c r="F9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="16" t="n"/>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="16" t="n"/>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="14" t="n"/>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="16" t="n"/>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
+      <c r="B11" s="14" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="16" t="n"/>
-      <c r="E12" s="16" t="n"/>
-      <c r="F12" s="16" t="n"/>
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="14" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -1233,178 +1208,167 @@
     <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>↑</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>End-2025 target status assessment and reporting (for reference)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="3" t="inlineStr">
+    <row r="1"/>
+    <row r="2" ht="39" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Your SR25 responses – Advancement, Communication and Marketing (AC&amp;M)</t>
         </is>
       </c>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="B3" s="18" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Your responses to the end-2025 reporting request, against the former Sustainability Plan 2030 (SP2030) targets. For reference only – please do not edit. Use the 'Back to request' links to return to the reporting template.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="B4" s="21" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>← Back to request</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="B5" s="22" t="inlineStr">
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Advancement, Communications &amp; Marketing</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="9" t="inlineStr">
+    <row r="6" ht="42" customHeight="1">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>SR25 ref</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>SP2030 target</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>2025 reporting request</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Confirmed end-2025 status</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>OPTION 1: Target-level reporting</t>
         </is>
       </c>
-      <c r="G6" s="9" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>OPTION 2: Indicator-level reporting</t>
         </is>
       </c>
-      <c r="H6" s="9" t="inlineStr">
+      <c r="H6" s="7" t="inlineStr">
         <is>
           <t>Supporting information/comments</t>
         </is>
       </c>
-      <c r="I6" s="9" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
         <is>
           <t>Related SR26 indicator(s)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="160" customHeight="1">
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>3e</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>The University has increased its engagement with alumni regarding sustainability</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="12" t="inlineStr">
         <is>
           <t>Annual climate and sustainability alumni community snapshot, including the number of related events and high-level audience demographics</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="12" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>A total of 1,947 alumni have attended one or more of the 70 climate or sustainability-related events so far this year, a small increase over the 2024 total.  Overall alumni engagement has declined slightly from last year, and so this result is encouraging.  Additional focus on impact in this space has been incorporated into the strategic planning activities for 2026 with the hopes of further widening and deepening engagement.</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr"/>
-      <c r="H7" s="14" t="inlineStr"/>
-      <c r="I7" s="14" t="inlineStr">
+      <c r="G7" s="12" t="inlineStr"/>
+      <c r="H7" s="12" t="inlineStr"/>
+      <c r="I7" s="12" t="inlineStr">
         <is>
           <t>EN1(c)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="160" customHeight="1">
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>4b(iii)</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>Graduates have increased capabilities to shape, lead and succeed in the careers, communities and industries of sustainable societies (year on year).</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
         <is>
           <t>Alumni Profile or case study demonstrating the impact our alumni have in sustainability is produced.</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>In the second half of 2025, there was 1 new article published on the Alumni website featuring University alumni that are having an impact on sustainability. The focus of the article was on nature and people and how the alum is helping to change behaviours to improve conservation efforts. The article was featured in the Alumni Newsletter and promoted on alumni social media.</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr"/>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="G8" s="12" t="inlineStr"/>
+      <c r="H8" s="12" t="inlineStr">
         <is>
           <t>https://www.unimelb.edu.au/alumni/stay-connected/news-and-stories/fast-five-with-whos-who-at-the-zoo</t>
         </is>
       </c>
-      <c r="I8" s="14" t="inlineStr"/>
-    </row>
-    <row r="9" ht="160" customHeight="1">
-      <c r="B9" s="12" t="inlineStr">
+      <c r="I8" s="12" t="inlineStr"/>
+    </row>
+    <row r="9" ht="409" customHeight="1">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>5b(ii)</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>The highest quality research is conducted that contributes to knowledge, action, and impact across the disciplinary and interdisciplinary dimensions of sustainability.</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Commentary on use of communication channels to disseminate sustainability-related research externally and the translation of sustainability-related research outcomes internally, drawing on Academic Division-level plans and varied cross-divisional activities and related outputs</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -1413,8 +1377,8 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr"/>
-      <c r="H9" s="14" t="inlineStr">
+      <c r="G9" s="12" t="inlineStr"/>
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -1427,7 +1391,7 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="I9" s="14" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
         <is>
           <t>TR2(a), CL2(c)</t>
         </is>
@@ -1450,10 +1414,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:E9"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="B1" t="inlineStr">
         <is>
           <t>(not used – no target status rating in 2026)</t>
@@ -1475,7 +1446,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="22" customHeight="1">
       <c r="B2" t="inlineStr">
         <is>
           <t>Please select from dropdown</t>
@@ -1497,7 +1468,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="22" customHeight="1">
       <c r="C3" t="inlineStr">
         <is>
           <t>No</t>
@@ -1514,7 +1485,7 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="22" customHeight="1">
       <c r="C4" t="inlineStr">
         <is>
           <t>Partially – see comments</t>
@@ -1531,35 +1502,35 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="22" customHeight="1">
       <c r="D5" t="inlineStr">
         <is>
           <t>Received</t>
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="22" customHeight="1">
       <c r="D6" t="inlineStr">
         <is>
           <t>First review</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="22" customHeight="1">
       <c r="D7" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="22" customHeight="1">
       <c r="D8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="22" customHeight="1">
       <c r="D9" t="inlineStr">
         <is>
           <t>Not required</t>

</xml_diff>

<commit_message>
v0.23: Rose feedback – due 24 Dec, request wording, EE1(b) dropped for ABP, P2 Gantt with governance deadlines, UoM banner and logo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
@@ -31,7 +31,7 @@
     <font>
       <name val="Aptos"/>
       <b val="1"/>
-      <color rgb="00002060"/>
+      <color rgb="00FFFFFF"/>
       <sz val="22"/>
     </font>
     <font>
@@ -110,7 +110,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +135,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00000F46"/>
       </patternFill>
     </fill>
   </fills>
@@ -170,9 +175,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="4"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -297,6 +305,96 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>57150</colOff>
+      <row>1</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>57150</colOff>
+      <row>1</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>57150</colOff>
+      <row>1</row>
+      <rowOff>57150</rowOff>
+    </from>
+    <ext cx="609600" cy="609600"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -588,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q20"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -608,24 +706,61 @@
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="20" customWidth="1" min="16" max="16"/>
     <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="39" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>SR26 sustainability reporting request</t>
         </is>
       </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>How to use this spreadsheet:</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>• For each row below, describe progress towards the target (Column L) and/or respond to the 2026 reporting request (Column M)
 • Provide supporting information if required (Column N), including links to documents or images
@@ -633,7 +768,7 @@
 • Where a related end-2025 target existed, click the ref in Column H to see your full SR25 response (Tab 3)
 • Use Tab 2 of this spreadsheet to highlight key sustainability stories (optional)
 • 2026 is a transition year: Sustainability 2030 launched ~20 October 2026, so report on activity across all of 2026 and any early actions since launch. No target status rating is requested this year.
-• Due: Tuesday 15 December 2026. Questions: Sustainability Strategy team (SST) – questions and clarifications are recorded centrally (contact email TBC); optional 1:1 meetings available on request</t>
+• Due: Thursday 24 December 2026 (Christmas shutdown). Questions: Sustainability Strategy team (SST) – questions and clarifications are recorded centrally (contact email TBC); optional 1:1 meetings available on request</t>
         </is>
       </c>
     </row>
@@ -644,7 +779,7 @@
     <row r="9"/>
     <row r="10"/>
     <row r="11" ht="39" customHeight="1">
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>AC&amp;M – Advancement, Communication and Marketing</t>
         </is>
@@ -652,190 +787,190 @@
     </row>
     <row r="12"/>
     <row r="13" ht="27" customHeight="1">
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Sustainability 2030 target and indicator</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>SR25 response</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr">
         <is>
           <t>End-2026 reporting (PLEASE COMPLETE THIS SECTION)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Ref</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Priority area</t>
         </is>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Sustainability 2030 target</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Indicator</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F14" s="8" t="inlineStr">
         <is>
           <t>2026 Reporting request</t>
         </is>
       </c>
-      <c r="G14" s="7" t="inlineStr">
+      <c r="G14" s="8" t="inlineStr">
         <is>
           <t>How SST will use this data</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="H14" s="8" t="inlineStr">
         <is>
           <t>Related SR25 ref</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="I14" s="8" t="inlineStr">
         <is>
           <t>End-2025 confirmed status</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="J14" s="8" t="inlineStr">
         <is>
           <t>End-2025 reporting response</t>
         </is>
       </c>
-      <c r="K14" s="7" t="inlineStr">
+      <c r="K14" s="8" t="inlineStr">
         <is>
           <t>Links and supporting information</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
+      <c r="L14" s="9" t="inlineStr">
         <is>
           <t>OPTION 1:  Target-level reporting (Column D)</t>
         </is>
       </c>
-      <c r="M14" s="8" t="inlineStr">
+      <c r="M14" s="9" t="inlineStr">
         <is>
           <t>OPTION 2:  Indicator level reporting (Column E/F)</t>
         </is>
       </c>
-      <c r="N14" s="8" t="inlineStr">
+      <c r="N14" s="9" t="inlineStr">
         <is>
           <t>Supporting information/comments</t>
         </is>
       </c>
-      <c r="O14" s="8" t="inlineStr">
+      <c r="O14" s="9" t="inlineStr">
         <is>
           <t>Data source and limitations</t>
         </is>
       </c>
-      <c r="P14" s="8" t="inlineStr">
+      <c r="P14" s="9" t="inlineStr">
         <is>
           <t>Data owner confirms information is accurate</t>
         </is>
       </c>
-      <c r="Q14" s="8" t="inlineStr">
+      <c r="Q14" s="9" t="inlineStr">
         <is>
           <t>Confirmed by (name, role, date)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="81" customHeight="1">
-      <c r="B15" s="9" t="inlineStr"/>
-      <c r="C15" s="9" t="inlineStr"/>
-      <c r="D15" s="9" t="inlineStr"/>
-      <c r="E15" s="9" t="inlineStr"/>
-      <c r="F15" s="9" t="inlineStr"/>
-      <c r="G15" s="9" t="inlineStr"/>
-      <c r="H15" s="9" t="inlineStr"/>
-      <c r="I15" s="9" t="inlineStr"/>
-      <c r="J15" s="9" t="inlineStr"/>
-      <c r="K15" s="9" t="inlineStr"/>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="B15" s="10" t="inlineStr"/>
+      <c r="C15" s="10" t="inlineStr"/>
+      <c r="D15" s="10" t="inlineStr"/>
+      <c r="E15" s="10" t="inlineStr"/>
+      <c r="F15" s="10" t="inlineStr"/>
+      <c r="G15" s="10" t="inlineStr"/>
+      <c r="H15" s="10" t="inlineStr"/>
+      <c r="I15" s="10" t="inlineStr"/>
+      <c r="J15" s="10" t="inlineStr"/>
+      <c r="K15" s="10" t="inlineStr"/>
+      <c r="L15" s="10" t="inlineStr">
         <is>
           <t>A general update on activities in relation to the overarching target (Column D)</t>
         </is>
       </c>
-      <c r="M15" s="9" t="inlineStr">
+      <c r="M15" s="10" t="inlineStr">
         <is>
           <t>Data and commentary in direct response to the reporting request (Column F)</t>
         </is>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="N15" s="10" t="inlineStr">
         <is>
           <t>Any additional information (e.g. links, images, documents)</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
+      <c r="O15" s="10" t="inlineStr">
         <is>
           <t>Where did this information come from (system, report, survey, person)? Note any gaps or limitations.</t>
         </is>
       </c>
-      <c r="P15" s="9" t="inlineStr">
+      <c r="P15" s="10" t="inlineStr">
         <is>
           <t>Select 'Yes' to confirm the information provided is accurate and can be used for reporting</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
+      <c r="Q15" s="10" t="inlineStr">
         <is>
           <t>Name, role and date of the person confirming</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="204" customHeight="1">
-      <c r="B16" s="10" t="inlineStr">
+    <row r="16" ht="171" customHeight="1">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>TR2(a)</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>Transformational research</t>
         </is>
       </c>
-      <c r="D16" s="11" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
         </is>
       </c>
-      <c r="E16" s="11" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
-Please provide examples of sustainability-related research impact from your Faculty/Portfolio across policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.</t>
-        </is>
-      </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from MRE.</t>
-        </is>
-      </c>
-      <c r="H16" s="13" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Please provide examples of sustainability-related research impact from your Faculty/Portfolio across policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.
+In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3).</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from Melbourne Research and Enterprise (MRE).</t>
+        </is>
+      </c>
+      <c r="H16" s="14" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I16" s="12" t="inlineStr">
+      <c r="I16" s="13" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J16" s="12" t="inlineStr">
+      <c r="J16" s="13" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -844,7 +979,7 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="K16" s="12" t="inlineStr">
+      <c r="K16" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -857,103 +992,103 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L16" s="14" t="n"/>
-      <c r="M16" s="14" t="n"/>
-      <c r="N16" s="14" t="n"/>
-      <c r="O16" s="14" t="n"/>
-      <c r="P16" s="14" t="n"/>
-      <c r="Q16" s="14" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="15" t="n"/>
+      <c r="N16" s="15" t="n"/>
+      <c r="O16" s="15" t="n"/>
+      <c r="P16" s="15" t="n"/>
+      <c r="Q16" s="15" t="n"/>
     </row>
     <row r="17" ht="150" customHeight="1">
-      <c r="B17" s="10" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>CL2(a)</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Climate leadership</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Develop understanding of our research and education programs that contribute to accelerating global decarbonisation and our own climate transition.</t>
         </is>
       </c>
-      <c r="E17" s="11" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>By 2028, develop and document institutional mapping of research and education activities that are designed to contribute to global decarbonisation</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Please list and describe examples of communications from your Faculty/Portfolio that demonstrate climate action, research and learning and aim to inform policy, sector or community decarbonisation efforts. Could include links, intended audiences and any available evidence of reach or influence.</t>
         </is>
       </c>
-      <c r="G17" s="12" t="inlineStr">
+      <c r="G17" s="13" t="inlineStr">
         <is>
           <t>We will use these examples to show how the University communicates climate research and learning to external audiences, and as an input to the institutional decarbonisation research and education mapping due by 2028.</t>
         </is>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>N/A – new indicator</t>
         </is>
       </c>
-      <c r="I17" s="12" t="inlineStr"/>
-      <c r="J17" s="12" t="inlineStr"/>
-      <c r="K17" s="12" t="inlineStr"/>
-      <c r="L17" s="14" t="n"/>
-      <c r="M17" s="14" t="n"/>
-      <c r="N17" s="14" t="n"/>
-      <c r="O17" s="14" t="n"/>
-      <c r="P17" s="14" t="n"/>
-      <c r="Q17" s="14" t="n"/>
-    </row>
-    <row r="18" ht="171" customHeight="1">
-      <c r="B18" s="10" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr"/>
+      <c r="J17" s="13" t="inlineStr"/>
+      <c r="K17" s="13" t="inlineStr"/>
+      <c r="L17" s="15" t="n"/>
+      <c r="M17" s="15" t="n"/>
+      <c r="N17" s="15" t="n"/>
+      <c r="O17" s="15" t="n"/>
+      <c r="P17" s="15" t="n"/>
+      <c r="Q17" s="15" t="n"/>
+    </row>
+    <row r="18" ht="150" customHeight="1">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>CL2(c)</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C18" s="12" t="inlineStr">
         <is>
           <t>Climate leadership</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Develop understanding of our research and education programs that contribute to accelerating global decarbonisation and our own climate transition.</t>
         </is>
       </c>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="E18" s="12" t="inlineStr">
         <is>
           <t>Ongoing communications that evidence the University’s climate action, research and learning to inform policy, sector and community decarbonisation efforts.</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
-List and describe communications from the faculty in terms of climate action, research and learning to inform policy, sector and community decarbonisation efforts</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>List and describe communications from the faculty in terms of climate action, research and learning to inform policy, sector and community decarbonisation efforts
+In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3).</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
         <is>
           <t>We will report on the University's ongoing climate communications in the Climate leadership section of the 2026 Sustainability Report, alongside contributions from Melbourne Climate Futures and the Melbourne Energy Institute.</t>
         </is>
       </c>
-      <c r="H18" s="13" t="inlineStr">
+      <c r="H18" s="14" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I18" s="12" t="inlineStr">
+      <c r="I18" s="13" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J18" s="12" t="inlineStr">
+      <c r="J18" s="13" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -962,7 +1097,7 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="K18" s="12" t="inlineStr">
+      <c r="K18" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -975,68 +1110,68 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L18" s="14" t="n"/>
-      <c r="M18" s="14" t="n"/>
-      <c r="N18" s="14" t="n"/>
-      <c r="O18" s="14" t="n"/>
-      <c r="P18" s="14" t="n"/>
-      <c r="Q18" s="14" t="n"/>
-    </row>
-    <row r="19" ht="188" customHeight="1">
-      <c r="B19" s="10" t="inlineStr">
+      <c r="L18" s="15" t="n"/>
+      <c r="M18" s="15" t="n"/>
+      <c r="N18" s="15" t="n"/>
+      <c r="O18" s="15" t="n"/>
+      <c r="P18" s="15" t="n"/>
+      <c r="Q18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="171" customHeight="1">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>EN1(c)</t>
         </is>
       </c>
-      <c r="C19" s="11" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>Enablers</t>
         </is>
       </c>
-      <c r="D19" s="11" t="inlineStr">
+      <c r="D19" s="12" t="inlineStr">
         <is>
           <t>Enablers</t>
         </is>
       </c>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>Coordinated internal engagement and external partnerships contributing to delivery of sustainability outcomes across priority areas.</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>In end-2025 reporting your area reported on the related SP2030 target 3e (click the ref in Column H to see it in full in Tab 3). Please build on this rather than repeating it, focusing on what is new in 2026.
-Please provide examples of internal engagement or external partnerships involving your Faculty/Portfolio that contributed to Sustainability 2030 outcomes, could include the priority area addressed, participating groups/partners, nature of the collaboration and key outcomes.</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Please provide examples of internal engagement or external partnerships involving your Faculty/Portfolio that contributed to Sustainability 2030 outcomes, could include the priority area addressed, participating groups/partners, nature of the collaboration and key outcomes.
+In end-2025 reporting your area reported on the related SP2030 target 3e (click the ref in Column H to see it in full in Tab 3).</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
         <is>
           <t>We will report on internal engagement and partnerships contributing to Sustainability 2030 outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
         </is>
       </c>
-      <c r="H19" s="13" t="inlineStr">
+      <c r="H19" s="14" t="inlineStr">
         <is>
           <t>3e
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I19" s="12" t="inlineStr">
+      <c r="I19" s="13" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J19" s="12" t="inlineStr">
+      <c r="J19" s="13" t="inlineStr">
         <is>
           <t>A total of 1,947 alumni have attended one or more of the 70 climate or sustainability-related events so far this year, a small increase over the 2024 total.  Overall alumni engagement has declined slightly from last year, and so this result is encouraging.  Additional focus on impact in this space has been incorporated into the strategic planning activities for 2026 with the hopes of further widening and deepening engagement.</t>
         </is>
       </c>
-      <c r="K19" s="12" t="inlineStr"/>
-      <c r="L19" s="14" t="n"/>
-      <c r="M19" s="14" t="n"/>
-      <c r="N19" s="14" t="n"/>
-      <c r="O19" s="14" t="n"/>
-      <c r="P19" s="14" t="n"/>
-      <c r="Q19" s="14" t="n"/>
+      <c r="K19" s="13" t="inlineStr"/>
+      <c r="L19" s="15" t="n"/>
+      <c r="M19" s="15" t="n"/>
+      <c r="N19" s="15" t="n"/>
+      <c r="O19" s="15" t="n"/>
+      <c r="P19" s="15" t="n"/>
+      <c r="Q19" s="15" t="n"/>
     </row>
     <row r="20"/>
   </sheetData>
@@ -1058,6 +1193,7 @@
     <hyperlink ref="H19" location="'3. SR25 responses'!B7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1067,7 +1203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1080,104 +1216,148 @@
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="39" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Highlighted stories (optional)</t>
         </is>
       </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
     </row>
     <row r="3"/>
     <row r="4"/>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>How to use this spreadsheet</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Please share up to 3 stories from 2026 which highlight your faculty's/portfolio's sustainability progress and/or impact. These stories can directly relate to Sustainability 2030 targets and indicators, or sustainability more generally. Due: Tuesday 15 December 2026 (early submission helps us develop case studies).</t>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Please share up to 3 stories from 2026 which highlight your faculty's/portfolio's sustainability progress and/or impact. These stories can directly relate to Sustainability 2030 targets and indicators, or sustainability more generally. Due: Thursday 24 December 2026 (Christmas shutdown) (early submission helps us develop case studies).</t>
         </is>
       </c>
     </row>
     <row r="6"/>
     <row r="7"/>
     <row r="8" ht="39" customHeight="1">
-      <c r="B8" s="17" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="C8" s="18" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="D8" s="17" t="inlineStr">
+      <c r="D8" s="18" t="inlineStr">
         <is>
           <t>Related Sustainability 2030 targets (optional)</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E8" s="18" t="inlineStr">
         <is>
           <t>Images and other media</t>
         </is>
       </c>
-      <c r="F8" s="17" t="inlineStr">
+      <c r="F8" s="18" t="inlineStr">
         <is>
           <t>Links and supporting documentation</t>
         </is>
       </c>
     </row>
     <row r="9" ht="90" customHeight="1">
-      <c r="B9" s="18" t="inlineStr"/>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr"/>
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>• Please include a brief description of a project or activity that has made a significant contribution to sustainability at the University (up to 250 words)
 • Summarise the benefits. Benefits may relate to operational outcomes, environmental/social outcomes, and sector benefits.</t>
         </is>
       </c>
-      <c r="D9" s="18" t="inlineStr"/>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="D9" s="19" t="inlineStr"/>
+      <c r="E9" s="19" t="inlineStr">
         <is>
           <t>(link to OneDrive/SharePoint files or published online content preferred)</t>
         </is>
       </c>
-      <c r="F9" s="18" t="inlineStr"/>
+      <c r="F9" s="19" t="inlineStr"/>
     </row>
     <row r="10" ht="120" customHeight="1">
       <c r="A10" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="15" t="n"/>
+      <c r="D11" s="15" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
+      <c r="B12" s="15" t="n"/>
+      <c r="C12" s="15" t="n"/>
+      <c r="D12" s="15" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
@@ -1185,6 +1365,7 @@
     <mergeCell ref="C5:F6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1194,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1206,169 +1387,214 @@
     <col width="60" customWidth="1" min="7" max="7"/>
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1"/>
-    <row r="2" ht="39" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="1" t="n"/>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+      <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
+      <c r="O1" s="1" t="n"/>
+      <c r="P1" s="1" t="n"/>
+      <c r="Q1" s="1" t="n"/>
+      <c r="R1" s="1" t="n"/>
+    </row>
+    <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="1" t="n"/>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Your SR25 responses – Advancement, Communication and Marketing (AC&amp;M)</t>
         </is>
       </c>
+      <c r="C2" s="1" t="n"/>
+      <c r="D2" s="1" t="n"/>
+      <c r="E2" s="1" t="n"/>
+      <c r="F2" s="1" t="n"/>
+      <c r="G2" s="1" t="n"/>
+      <c r="H2" s="1" t="n"/>
+      <c r="I2" s="1" t="n"/>
+      <c r="J2" s="1" t="n"/>
+      <c r="K2" s="1" t="n"/>
+      <c r="L2" s="1" t="n"/>
+      <c r="M2" s="1" t="n"/>
+      <c r="N2" s="1" t="n"/>
+      <c r="O2" s="1" t="n"/>
+      <c r="P2" s="1" t="n"/>
+      <c r="Q2" s="1" t="n"/>
+      <c r="R2" s="1" t="n"/>
     </row>
     <row r="3" ht="32" customHeight="1">
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Your responses to the end-2025 reporting request, against the former Sustainability Plan 2030 (SP2030) targets. For reference only – please do not edit. Use the 'Back to request' links to return to the reporting template.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="B4" s="19" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>← Back to request</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Advancement, Communications &amp; Marketing</t>
         </is>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1">
-      <c r="B6" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>SR25 ref</t>
         </is>
       </c>
-      <c r="C6" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>SP2030 target</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>2025 reporting request</t>
         </is>
       </c>
-      <c r="E6" s="7" t="inlineStr">
+      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Confirmed end-2025 status</t>
         </is>
       </c>
-      <c r="F6" s="7" t="inlineStr">
+      <c r="F6" s="8" t="inlineStr">
         <is>
           <t>OPTION 1: Target-level reporting</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>OPTION 2: Indicator-level reporting</t>
         </is>
       </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>Supporting information/comments</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Related SR26 indicator(s)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="160" customHeight="1">
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>3e</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>The University has increased its engagement with alumni regarding sustainability</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Annual climate and sustainability alumni community snapshot, including the number of related events and high-level audience demographics</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>A total of 1,947 alumni have attended one or more of the 70 climate or sustainability-related events so far this year, a small increase over the 2024 total.  Overall alumni engagement has declined slightly from last year, and so this result is encouraging.  Additional focus on impact in this space has been incorporated into the strategic planning activities for 2026 with the hopes of further widening and deepening engagement.</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr"/>
-      <c r="H7" s="12" t="inlineStr"/>
-      <c r="I7" s="12" t="inlineStr">
+      <c r="G7" s="13" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr"/>
+      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>EN1(c)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="160" customHeight="1">
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>4b(iii)</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Graduates have increased capabilities to shape, lead and succeed in the careers, communities and industries of sustainable societies (year on year).</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>Alumni Profile or case study demonstrating the impact our alumni have in sustainability is produced.</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>In the second half of 2025, there was 1 new article published on the Alumni website featuring University alumni that are having an impact on sustainability. The focus of the article was on nature and people and how the alum is helping to change behaviours to improve conservation efforts. The article was featured in the Alumni Newsletter and promoted on alumni social media.</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr"/>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="G8" s="13" t="inlineStr"/>
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>https://www.unimelb.edu.au/alumni/stay-connected/news-and-stories/fast-five-with-whos-who-at-the-zoo</t>
         </is>
       </c>
-      <c r="I8" s="12" t="inlineStr"/>
+      <c r="I8" s="13" t="inlineStr"/>
     </row>
     <row r="9" ht="409" customHeight="1">
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>5b(ii)</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>The highest quality research is conducted that contributes to knowledge, action, and impact across the disciplinary and interdisciplinary dimensions of sustainability.</t>
         </is>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Commentary on use of communication channels to disseminate sustainability-related research externally and the translation of sustainability-related research outcomes internally, drawing on Academic Division-level plans and varied cross-divisional activities and related outputs</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -1377,8 +1603,8 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr"/>
-      <c r="H9" s="12" t="inlineStr">
+      <c r="G9" s="13" t="inlineStr"/>
+      <c r="H9" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -1391,7 +1617,7 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="I9" s="12" t="inlineStr">
+      <c r="I9" s="13" t="inlineStr">
         <is>
           <t>TR2(a), CL2(c)</t>
         </is>
@@ -1405,6 +1631,7 @@
     <hyperlink ref="B4" location="'1. Reporting template'!A1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
v0.26: Rose feedback on MRE, CI&S, CFOG, AC&M; remove owner-confirm columns; per-unit wording; master wording linked to request files
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PXuBp5SMoG4pD1jWH8rtoe
</commit_message>
<xml_diff>
--- a/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
+++ b/output/central_unit_requests/ACM - SR26 sustainability reporting request.xlsx
@@ -212,12 +212,12 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
       <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -703,9 +703,9 @@
     <col width="48" customWidth="1" min="12" max="12"/>
     <col width="48" customWidth="1" min="13" max="13"/>
     <col width="30" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
@@ -764,7 +764,8 @@
         <is>
           <t>• For each row below, describe progress towards the target (Column L) and/or respond to the 2026 reporting request (Column M)
 • Provide supporting information if required (Column N), including links to documents or images
-• Note the source of your information and any limitations (Column O), then confirm the information is accurate (Columns P–Q)
+• Note the source of your information, any limitations and the person closest to the data (Column O)
+• Please return the spreadsheet once it has been reviewed and confirmed by your area's senior lead
 • Where a related end-2025 target existed, click the ref in Column H to see your full SR25 response (Tab 3)
 • Use Tab 2 of this spreadsheet to highlight key sustainability stories (optional)
 • 2026 is a transition year: Sustainability 2030 launched ~20 October 2026, so report on activity across all of 2026 and any early actions since launch. No target status rating is requested this year.
@@ -803,7 +804,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="42" customHeight="1">
       <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Ref</t>
@@ -871,17 +872,7 @@
       </c>
       <c r="O14" s="9" t="inlineStr">
         <is>
-          <t>Data source and limitations</t>
-        </is>
-      </c>
-      <c r="P14" s="9" t="inlineStr">
-        <is>
-          <t>Data owner confirms information is accurate</t>
-        </is>
-      </c>
-      <c r="Q14" s="9" t="inlineStr">
-        <is>
-          <t>Confirmed by (name, role, date)</t>
+          <t>Data source, limitations and contact person</t>
         </is>
       </c>
     </row>
@@ -913,64 +904,98 @@
       </c>
       <c r="O15" s="10" t="inlineStr">
         <is>
-          <t>Where did this information come from (system, report, survey, person)? Note any gaps or limitations.</t>
-        </is>
-      </c>
-      <c r="P15" s="10" t="inlineStr">
-        <is>
-          <t>Select 'Yes' to confirm the information provided is accurate and can be used for reporting</t>
-        </is>
-      </c>
-      <c r="Q15" s="10" t="inlineStr">
-        <is>
-          <t>Name, role and date of the person confirming</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="171" customHeight="1">
+          <t>Where did this information come from (system, report, survey)? Note any gaps or limitations, and the person closest to the data we can follow up with.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="150" customHeight="1">
       <c r="B16" s="11" t="inlineStr">
         <is>
+          <t>EE1(d)</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Exceptional education</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Provide our students with learning experiences that help them build the knowledge, skills and relationships to lead change for sustainable societies.</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Alumni profiles demonstrating how graduates contribute to sustainability through their careers or communities.</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Can you list any notable alumni working in sustainability? (Name, course and graduating year, a short summary and a link to a profile if available; please note whether consent to be featured is likely.)</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>We will use nominated alumni to develop short graduate profiles for the 2026 Sustainability Report (subject to consent), and record any faculty approaches to tracking graduate outcomes to inform how this indicator is measured from 2027.</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>N/A – new indicator</t>
+        </is>
+      </c>
+      <c r="I16" s="13" t="inlineStr"/>
+      <c r="J16" s="13" t="inlineStr"/>
+      <c r="K16" s="13" t="inlineStr"/>
+      <c r="L16" s="14" t="n"/>
+      <c r="M16" s="14" t="n"/>
+      <c r="N16" s="14" t="n"/>
+      <c r="O16" s="14" t="n"/>
+    </row>
+    <row r="17" ht="171" customHeight="1">
+      <c r="B17" s="11" t="inlineStr">
+        <is>
           <t>TR2(a)</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Transformational research</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Deliver high-quality research and partnerships that contribute to sustainability outcomes and demonstrable societal benefit.</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E17" s="12" t="inlineStr">
         <is>
           <t>Evidence of sustainability-related research impact across diverse pathways, could include policy, industry, community, practice, cultural and institutional outcomes</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>Please provide examples of sustainability-related research impact from your Faculty/Portfolio across policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Please provide examples of sustainability-related research impact from across the University in policy, industry, community, practice, cultural or institutional pathways. For key examples, briefly describe the research contribution, partner/user and resulting outcome or influence.
 In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="G17" s="13" t="inlineStr">
         <is>
           <t>We will collate research impact examples across faculties to show the breadth of sustainability-related research impact in the Transformational research section of the 2026 Sustainability Report, complementing University-wide metrics from Melbourne Research and Enterprise (MRE).</t>
         </is>
       </c>
-      <c r="H16" s="14" t="inlineStr">
+      <c r="H17" s="15" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
         </is>
       </c>
-      <c r="I16" s="13" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>Met or exceeded</t>
         </is>
       </c>
-      <c r="J16" s="13" t="inlineStr">
+      <c r="J17" s="13" t="inlineStr">
         <is>
           <t>https://pursuit.unimelb.edu.au/articles/the-worlds-most-powerful-ocean-current-could-slow-by-2050
 In July 2025, the University launched its new research strategy, Advancing Research 2030: Excellence for Impact. This strategy introduced a new research impact accelerator, Climate sustainability and ecosystem health, to enable focus and partnership on research helping to address climate change and sustainability challenges. This theme was highlighted at the University’s inaugural Open Day 2025 ‘Research at Melbourne’ pavilion, which featured research on Indigenous water rights, Corroboree frog conservation and a multimedia bushfire simulation called ‘Flashover’. 
@@ -979,7 +1004,7 @@
 But our biggest story of the year was the awarding of the Nobel Prize in Chemistry to Professor Richard Robson for the development of metal-organic frameworks, a new class of materials that could be crucial to the energy revolution and a low-carbon future.</t>
         </is>
       </c>
-      <c r="K16" s="13" t="inlineStr">
+      <c r="K17" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">
 https://research.unimelb.edu.au/strengths/advancing-research-2030-excellence-for-impact
@@ -992,58 +1017,10 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L16" s="15" t="n"/>
-      <c r="M16" s="15" t="n"/>
-      <c r="N16" s="15" t="n"/>
-      <c r="O16" s="15" t="n"/>
-      <c r="P16" s="15" t="n"/>
-      <c r="Q16" s="15" t="n"/>
-    </row>
-    <row r="17" ht="150" customHeight="1">
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>CL2(a)</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Climate leadership</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Develop understanding of our research and education programs that contribute to accelerating global decarbonisation and our own climate transition.</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
-        <is>
-          <t>By 2028, develop and document institutional mapping of research and education activities that are designed to contribute to global decarbonisation</t>
-        </is>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
-        <is>
-          <t>Please list and describe examples of communications from your Faculty/Portfolio that demonstrate climate action, research and learning and aim to inform policy, sector or community decarbonisation efforts. Could include links, intended audiences and any available evidence of reach or influence.</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="inlineStr">
-        <is>
-          <t>We will use these examples to show how the University communicates climate research and learning to external audiences, and as an input to the institutional decarbonisation research and education mapping due by 2028.</t>
-        </is>
-      </c>
-      <c r="H17" s="13" t="inlineStr">
-        <is>
-          <t>N/A – new indicator</t>
-        </is>
-      </c>
-      <c r="I17" s="13" t="inlineStr"/>
-      <c r="J17" s="13" t="inlineStr"/>
-      <c r="K17" s="13" t="inlineStr"/>
-      <c r="L17" s="15" t="n"/>
-      <c r="M17" s="15" t="n"/>
-      <c r="N17" s="15" t="n"/>
-      <c r="O17" s="15" t="n"/>
-      <c r="P17" s="15" t="n"/>
-      <c r="Q17" s="15" t="n"/>
+      <c r="L17" s="14" t="n"/>
+      <c r="M17" s="14" t="n"/>
+      <c r="N17" s="14" t="n"/>
+      <c r="O17" s="14" t="n"/>
     </row>
     <row r="18" ht="150" customHeight="1">
       <c r="B18" s="11" t="inlineStr">
@@ -1068,7 +1045,7 @@
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>List and describe communications from the faculty in terms of climate action, research and learning to inform policy, sector and community decarbonisation efforts
+          <t>List and describe communications from across the University in terms of climate action, research and learning to inform policy, sector and community decarbonisation efforts
 In end-2025 reporting your area reported on the related SP2030 target 5b(ii) (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
@@ -1077,7 +1054,7 @@
           <t>We will report on the University's ongoing climate communications in the Climate leadership section of the 2026 Sustainability Report, alongside contributions from Melbourne Climate Futures and the Melbourne Energy Institute.</t>
         </is>
       </c>
-      <c r="H18" s="14" t="inlineStr">
+      <c r="H18" s="15" t="inlineStr">
         <is>
           <t>5b(ii)
 → view SR25 response</t>
@@ -1110,14 +1087,12 @@
 https://pursuit.unimelb.edu.au/articles/australias-largest-pharmaceutical-companies-need-to-do-more-to-reduce-their-carbon-footprint</t>
         </is>
       </c>
-      <c r="L18" s="15" t="n"/>
-      <c r="M18" s="15" t="n"/>
-      <c r="N18" s="15" t="n"/>
-      <c r="O18" s="15" t="n"/>
-      <c r="P18" s="15" t="n"/>
-      <c r="Q18" s="15" t="n"/>
-    </row>
-    <row r="19" ht="171" customHeight="1">
+      <c r="L18" s="14" t="n"/>
+      <c r="M18" s="14" t="n"/>
+      <c r="N18" s="14" t="n"/>
+      <c r="O18" s="14" t="n"/>
+    </row>
+    <row r="19" ht="154" customHeight="1">
       <c r="B19" s="11" t="inlineStr">
         <is>
           <t>EN1(c)</t>
@@ -1140,16 +1115,16 @@
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Please provide examples of internal engagement or external partnerships involving your Faculty/Portfolio that contributed to Sustainability 2030 outcomes, could include the priority area addressed, participating groups/partners, nature of the collaboration and key outcomes.
+          <t>Please provide examples of internal engagement or external partnerships involving the University that contributed to sustainability outcomes, could include the priority area addressed, participating groups/partners, nature of the collaboration and key outcomes.
 In end-2025 reporting your area reported on the related SP2030 target 3e (click the ref in Column H to see it in full in Tab 3).</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>We will report on internal engagement and partnerships contributing to Sustainability 2030 outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
-        </is>
-      </c>
-      <c r="H19" s="14" t="inlineStr">
+          <t>We will report on internal engagement and partnerships contributing to sustainability outcomes, and update our record of sustainability-focused communities of practice and contacts across the University.</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
         <is>
           <t>3e
 → view SR25 response</t>
@@ -1166,29 +1141,22 @@
         </is>
       </c>
       <c r="K19" s="13" t="inlineStr"/>
-      <c r="L19" s="15" t="n"/>
-      <c r="M19" s="15" t="n"/>
-      <c r="N19" s="15" t="n"/>
-      <c r="O19" s="15" t="n"/>
-      <c r="P19" s="15" t="n"/>
-      <c r="Q19" s="15" t="n"/>
+      <c r="L19" s="14" t="n"/>
+      <c r="M19" s="14" t="n"/>
+      <c r="N19" s="14" t="n"/>
+      <c r="O19" s="14" t="n"/>
     </row>
     <row r="20"/>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>
   <mergeCells count="4">
     <mergeCell ref="C13:G13"/>
-    <mergeCell ref="L13:Q13"/>
+    <mergeCell ref="L13:O13"/>
     <mergeCell ref="D4:G8"/>
     <mergeCell ref="B4:C8"/>
   </mergeCells>
-  <dataValidations count="1">
-    <dataValidation sqref="P16:P19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid entry" error="Please select from the dropdown" type="list">
-      <formula1>=Lists!$C$2:$C$4</formula1>
-    </dataValidation>
-  </dataValidations>
   <hyperlinks>
-    <hyperlink ref="H16" location="'3. SR25 responses'!B9"/>
+    <hyperlink ref="H17" location="'3. SR25 responses'!B9"/>
     <hyperlink ref="H18" location="'3. SR25 responses'!B9"/>
     <hyperlink ref="H19" location="'3. SR25 responses'!B7"/>
   </hyperlinks>
@@ -1333,31 +1301,31 @@
       <c r="A10" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="14" t="n"/>
+      <c r="F10" s="14" t="n"/>
     </row>
     <row r="11" ht="120" customHeight="1">
       <c r="A11" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="15" t="n"/>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
+      <c r="B11" s="14" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n"/>
     </row>
     <row r="12" ht="120" customHeight="1">
       <c r="A12" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="15" t="n"/>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
+      <c r="B12" s="14" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="14" t="n"/>
+      <c r="F12" s="14" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="0" sort="1"/>

</xml_diff>